<commit_message>
Sync review data 2026-10-10
</commit_message>
<xml_diff>
--- a/review-results/复盘信息抓取-20261010.xlsx
+++ b/review-results/复盘信息抓取-20261010.xlsx
@@ -5113,8 +5113,27 @@
       </c>
     </row>
     <row r="2">
-      <c r="D2" s="3" t="n"/>
-      <c r="E2" s="3" t="n"/>
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>现货实时交易价格曲线</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="n">
+        <v>13153.599</v>
+      </c>
+      <c r="E2" s="3" t="n">
+        <v>382.81</v>
+      </c>
       <c r="H2" t="inlineStr">
         <is>
           <t>现货日前交易价格曲线</t>
@@ -5138,8 +5157,27 @@
       </c>
     </row>
     <row r="3">
-      <c r="D3" s="3" t="n"/>
-      <c r="E3" s="3" t="n"/>
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>现货实时交易价格曲线</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>02</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="n">
+        <v>12468.143</v>
+      </c>
+      <c r="E3" s="3" t="n">
+        <v>361.5</v>
+      </c>
       <c r="H3" t="inlineStr">
         <is>
           <t>现货日前交易价格曲线</t>
@@ -5163,8 +5201,27 @@
       </c>
     </row>
     <row r="4">
-      <c r="D4" s="3" t="n"/>
-      <c r="E4" s="3" t="n"/>
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>现货实时交易价格曲线</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>03</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="n">
+        <v>14680.228</v>
+      </c>
+      <c r="E4" s="3" t="n">
+        <v>384.403</v>
+      </c>
       <c r="H4" t="inlineStr">
         <is>
           <t>现货日前交易价格曲线</t>
@@ -5188,8 +5245,27 @@
       </c>
     </row>
     <row r="5">
-      <c r="D5" s="3" t="n"/>
-      <c r="E5" s="3" t="n"/>
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>现货实时交易价格曲线</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>04</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="n">
+        <v>14081.336</v>
+      </c>
+      <c r="E5" s="3" t="n">
+        <v>432.223</v>
+      </c>
       <c r="H5" t="inlineStr">
         <is>
           <t>现货日前交易价格曲线</t>
@@ -5213,8 +5289,27 @@
       </c>
     </row>
     <row r="6">
-      <c r="D6" s="3" t="n"/>
-      <c r="E6" s="3" t="n"/>
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>现货实时交易价格曲线</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>05</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="n">
+        <v>13861.699</v>
+      </c>
+      <c r="E6" s="3" t="n">
+        <v>455.298</v>
+      </c>
       <c r="H6" t="inlineStr">
         <is>
           <t>现货日前交易价格曲线</t>
@@ -5238,8 +5333,27 @@
       </c>
     </row>
     <row r="7">
-      <c r="D7" s="3" t="n"/>
-      <c r="E7" s="3" t="n"/>
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>现货实时交易价格曲线</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>06</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="n">
+        <v>14581.614</v>
+      </c>
+      <c r="E7" s="3" t="n">
+        <v>409.633</v>
+      </c>
       <c r="H7" t="inlineStr">
         <is>
           <t>现货日前交易价格曲线</t>
@@ -5263,8 +5377,27 @@
       </c>
     </row>
     <row r="8">
-      <c r="D8" s="3" t="n"/>
-      <c r="E8" s="3" t="n"/>
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>现货实时交易价格曲线</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>07</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="n">
+        <v>15427.314</v>
+      </c>
+      <c r="E8" s="3" t="n">
+        <v>405.15</v>
+      </c>
       <c r="H8" t="inlineStr">
         <is>
           <t>现货日前交易价格曲线</t>
@@ -5288,8 +5421,27 @@
       </c>
     </row>
     <row r="9">
-      <c r="D9" s="3" t="n"/>
-      <c r="E9" s="3" t="n"/>
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>现货实时交易价格曲线</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>08</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="n">
+        <v>16386.34</v>
+      </c>
+      <c r="E9" s="3" t="n">
+        <v>364.003</v>
+      </c>
       <c r="H9" t="inlineStr">
         <is>
           <t>现货日前交易价格曲线</t>
@@ -5313,8 +5465,27 @@
       </c>
     </row>
     <row r="10">
-      <c r="D10" s="3" t="n"/>
-      <c r="E10" s="3" t="n"/>
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>现货实时交易价格曲线</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>09</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="n">
+        <v>15713.41</v>
+      </c>
+      <c r="E10" s="3" t="n">
+        <v>324.23</v>
+      </c>
       <c r="H10" t="inlineStr">
         <is>
           <t>现货日前交易价格曲线</t>
@@ -5338,8 +5509,27 @@
       </c>
     </row>
     <row r="11">
-      <c r="D11" s="3" t="n"/>
-      <c r="E11" s="3" t="n"/>
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>现货实时交易价格曲线</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="n">
+        <v>16617.163</v>
+      </c>
+      <c r="E11" s="3" t="n">
+        <v>299.71</v>
+      </c>
       <c r="H11" t="inlineStr">
         <is>
           <t>现货日前交易价格曲线</t>
@@ -5363,8 +5553,27 @@
       </c>
     </row>
     <row r="12">
-      <c r="D12" s="3" t="n"/>
-      <c r="E12" s="3" t="n"/>
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>现货实时交易价格曲线</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="n">
+        <v>18511.442</v>
+      </c>
+      <c r="E12" s="3" t="n">
+        <v>317.293</v>
+      </c>
       <c r="H12" t="inlineStr">
         <is>
           <t>现货日前交易价格曲线</t>
@@ -5388,8 +5597,27 @@
       </c>
     </row>
     <row r="13">
-      <c r="D13" s="3" t="n"/>
-      <c r="E13" s="3" t="n"/>
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>现货实时交易价格曲线</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="n">
+        <v>18961.52</v>
+      </c>
+      <c r="E13" s="3" t="n">
+        <v>290.22</v>
+      </c>
       <c r="H13" t="inlineStr">
         <is>
           <t>现货日前交易价格曲线</t>
@@ -5413,8 +5641,27 @@
       </c>
     </row>
     <row r="14">
-      <c r="D14" s="3" t="n"/>
-      <c r="E14" s="3" t="n"/>
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>现货实时交易价格曲线</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="D14" s="3" t="n">
+        <v>18543.915</v>
+      </c>
+      <c r="E14" s="3" t="n">
+        <v>309.56</v>
+      </c>
       <c r="H14" t="inlineStr">
         <is>
           <t>现货日前交易价格曲线</t>
@@ -5438,8 +5685,27 @@
       </c>
     </row>
     <row r="15">
-      <c r="D15" s="3" t="n"/>
-      <c r="E15" s="3" t="n"/>
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>现货实时交易价格曲线</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="n">
+        <v>17904.954</v>
+      </c>
+      <c r="E15" s="3" t="n">
+        <v>307.798</v>
+      </c>
       <c r="H15" t="inlineStr">
         <is>
           <t>现货日前交易价格曲线</t>
@@ -5463,8 +5729,27 @@
       </c>
     </row>
     <row r="16">
-      <c r="D16" s="3" t="n"/>
-      <c r="E16" s="3" t="n"/>
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>现货实时交易价格曲线</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="D16" s="3" t="n">
+        <v>17720.985</v>
+      </c>
+      <c r="E16" s="3" t="n">
+        <v>346.603</v>
+      </c>
       <c r="H16" t="inlineStr">
         <is>
           <t>现货日前交易价格曲线</t>
@@ -5488,8 +5773,27 @@
       </c>
     </row>
     <row r="17">
-      <c r="D17" s="3" t="n"/>
-      <c r="E17" s="3" t="n"/>
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>现货实时交易价格曲线</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="D17" s="3" t="n">
+        <v>17134.574</v>
+      </c>
+      <c r="E17" s="3" t="n">
+        <v>427.643</v>
+      </c>
       <c r="H17" t="inlineStr">
         <is>
           <t>现货日前交易价格曲线</t>
@@ -5513,8 +5817,27 @@
       </c>
     </row>
     <row r="18">
-      <c r="D18" s="3" t="n"/>
-      <c r="E18" s="3" t="n"/>
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>现货实时交易价格曲线</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>17</t>
+        </is>
+      </c>
+      <c r="D18" s="3" t="n">
+        <v>17202.668</v>
+      </c>
+      <c r="E18" s="3" t="n">
+        <v>472.67</v>
+      </c>
       <c r="H18" t="inlineStr">
         <is>
           <t>现货日前交易价格曲线</t>
@@ -5538,8 +5861,27 @@
       </c>
     </row>
     <row r="19">
-      <c r="D19" s="3" t="n"/>
-      <c r="E19" s="3" t="n"/>
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>现货实时交易价格曲线</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="D19" s="3" t="n">
+        <v>16952.251</v>
+      </c>
+      <c r="E19" s="3" t="n">
+        <v>444.943</v>
+      </c>
       <c r="H19" t="inlineStr">
         <is>
           <t>现货日前交易价格曲线</t>
@@ -5563,8 +5905,27 @@
       </c>
     </row>
     <row r="20">
-      <c r="D20" s="3" t="n"/>
-      <c r="E20" s="3" t="n"/>
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>现货实时交易价格曲线</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="D20" s="3" t="n">
+        <v>15985.16</v>
+      </c>
+      <c r="E20" s="3" t="n">
+        <v>448.06</v>
+      </c>
       <c r="H20" t="inlineStr">
         <is>
           <t>现货日前交易价格曲线</t>
@@ -5588,8 +5949,27 @@
       </c>
     </row>
     <row r="21">
-      <c r="D21" s="3" t="n"/>
-      <c r="E21" s="3" t="n"/>
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>现货实时交易价格曲线</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="D21" s="3" t="n">
+        <v>13688.886</v>
+      </c>
+      <c r="E21" s="3" t="n">
+        <v>417.553</v>
+      </c>
       <c r="H21" t="inlineStr">
         <is>
           <t>现货日前交易价格曲线</t>
@@ -5613,8 +5993,27 @@
       </c>
     </row>
     <row r="22">
-      <c r="D22" s="3" t="n"/>
-      <c r="E22" s="3" t="n"/>
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>现货实时交易价格曲线</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>21</t>
+        </is>
+      </c>
+      <c r="D22" s="3" t="n">
+        <v>13291.937</v>
+      </c>
+      <c r="E22" s="3" t="n">
+        <v>440.923</v>
+      </c>
       <c r="H22" t="inlineStr">
         <is>
           <t>现货日前交易价格曲线</t>
@@ -5638,8 +6037,27 @@
       </c>
     </row>
     <row r="23">
-      <c r="D23" s="3" t="n"/>
-      <c r="E23" s="3" t="n"/>
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>现货实时交易价格曲线</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>22</t>
+        </is>
+      </c>
+      <c r="D23" s="3" t="n">
+        <v>13734.692</v>
+      </c>
+      <c r="E23" s="3" t="n">
+        <v>453.845</v>
+      </c>
       <c r="H23" t="inlineStr">
         <is>
           <t>现货日前交易价格曲线</t>
@@ -5663,8 +6081,27 @@
       </c>
     </row>
     <row r="24">
-      <c r="D24" s="3" t="n"/>
-      <c r="E24" s="3" t="n"/>
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>现货实时交易价格曲线</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>23</t>
+        </is>
+      </c>
+      <c r="D24" s="3" t="n">
+        <v>13472.585</v>
+      </c>
+      <c r="E24" s="3" t="n">
+        <v>441.078</v>
+      </c>
       <c r="H24" t="inlineStr">
         <is>
           <t>现货日前交易价格曲线</t>
@@ -5688,8 +6125,27 @@
       </c>
     </row>
     <row r="25">
-      <c r="D25" s="3" t="n"/>
-      <c r="E25" s="3" t="n"/>
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>现货实时交易价格曲线</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
+      <c r="D25" s="3" t="n">
+        <v>13785.327</v>
+      </c>
+      <c r="E25" s="3" t="n">
+        <v>449.465</v>
+      </c>
       <c r="H25" t="inlineStr">
         <is>
           <t>现货日前交易价格曲线</t>
@@ -16831,7 +17287,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>现货日前交易价格曲线</t>
+          <t>现货实时交易价格曲线</t>
         </is>
       </c>
       <c r="B2" t="n">
@@ -16844,46 +17300,46 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>非市场化机组总出力</t>
+          <t>现货日前交易价格曲线</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>96</v>
+        <v>24</v>
       </c>
       <c r="C3" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>新能源实际发电曲线</t>
+          <t>非市场化机组总出力</t>
         </is>
       </c>
       <c r="B4" t="n">
         <v>96</v>
       </c>
       <c r="C4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>实际系统负荷</t>
+          <t>新能源实际发电曲线</t>
         </is>
       </c>
       <c r="B5" t="n">
         <v>96</v>
       </c>
       <c r="C5" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>省间联络线输电情况</t>
+          <t>实际系统负荷</t>
         </is>
       </c>
       <c r="B6" t="n">
@@ -16896,24 +17352,24 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>各时段各类电源电量</t>
+          <t>省间联络线输电情况</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>960</v>
+        <v>96</v>
       </c>
       <c r="C7" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>各时段各类电源的开机台数</t>
+          <t>各时段各类电源电量</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>768</v>
+        <v>960</v>
       </c>
       <c r="C8" t="n">
         <v>5</v>
@@ -16922,30 +17378,42 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>实时储能充电计划及电价</t>
+          <t>各时段各类电源的开机台数</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>96</v>
+        <v>768</v>
       </c>
       <c r="C9" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>日前储能充电计划及电价</t>
+          <t>实时储能充电计划及电价</t>
         </is>
       </c>
       <c r="B10" t="n">
         <v>96</v>
       </c>
       <c r="C10" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>日前储能充电计划及电价</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>96</v>
+      </c>
+      <c r="C11" t="n">
         <v>8</v>
       </c>
     </row>
-    <row r="11"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>